<commit_message>
ATRG v2: HOD approvals, report templates as data, Gemini document intake
- HOD portal, approval workflow, sealed records, field registry and versioned report templates
- Unified document reading (PDF, photo, Excel in any layout, CSV) with Gemini at every upload point,
  side-by-side review, confirm all, clear auto-filled values; own Excel templates read without AI
- Verify / lock with missing values (reason recorded in the activity log)
- manage.py check-ai, tools/ai_accuracy.py (docs/ai_accuracy.md), intake and workflow tests

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/customer_request_filled.xlsx
+++ b/sample_data/customer_request_filled.xlsx
@@ -580,7 +580,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>1. Customer &amp; sample (Request form - sheet 1)</t>
+          <t>Request form - Sheet 1</t>
         </is>
       </c>
     </row>
@@ -825,7 +825,7 @@
     <row r="25">
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>2. Request form - sheet 2</t>
+          <t>Request form - Sheet 2</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -883,7 +883,7 @@
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>3. Proforma for transformers (manufacturer-declared data)</t>
+          <t>Proforma for transformers</t>
         </is>
       </c>
     </row>

</xml_diff>